<commit_message>
feat: new order summary table, PDF with unit column, fix confirm view flow
</commit_message>
<xml_diff>
--- a/public/clientes.xlsx
+++ b/public/clientes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yeres\OneDrive\Documentos\Webs\PREVENA PG\Skills\PreventaPG\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D2A4443-85B5-4F68-8F71-58705F6D8EA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B006F855-34D4-4D6A-86A3-6F420B5EABAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="40">
   <si>
     <t>Cliente</t>
   </si>
@@ -70,14 +70,97 @@
   </si>
   <si>
     <t>Raul Peña Cornejo</t>
+  </si>
+  <si>
+    <t>Mari Machare</t>
+  </si>
+  <si>
+    <t>Rosa Temoche Arca</t>
+  </si>
+  <si>
+    <t>Sandra Vinces Timana</t>
+  </si>
+  <si>
+    <t>Talara - Tablaso</t>
+  </si>
+  <si>
+    <t>Talara - Serpetro</t>
+  </si>
+  <si>
+    <t>Talara  - Acapulco</t>
+  </si>
+  <si>
+    <t>Nair Romero Nole</t>
+  </si>
+  <si>
+    <t>Aide Nole</t>
+  </si>
+  <si>
+    <t>Yanina Bocanegra</t>
+  </si>
+  <si>
+    <t>Sandra Alburqueue</t>
+  </si>
+  <si>
+    <t>Mercedes Amaya</t>
+  </si>
+  <si>
+    <t>Luis Marques Alama</t>
+  </si>
+  <si>
+    <t>Esterfilia</t>
+  </si>
+  <si>
+    <t>Nelly Vite Villegas</t>
+  </si>
+  <si>
+    <t>Roccio Romero Nole</t>
+  </si>
+  <si>
+    <t>Rosendo Peña</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Maria Huamanga </t>
+  </si>
+  <si>
+    <t>Talara - Central</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yobani </t>
+  </si>
+  <si>
+    <t>Elmer Raul</t>
+  </si>
+  <si>
+    <t>Miñope</t>
+  </si>
+  <si>
+    <t>Boris</t>
+  </si>
+  <si>
+    <t>Canales Ojeda</t>
+  </si>
+  <si>
+    <t>Prado</t>
+  </si>
+  <si>
+    <t>Talara - Parada</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -105,8 +188,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -387,11 +471,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="35.33203125" customWidth="1"/>
-    <col min="2" max="2" width="35.44140625" customWidth="1"/>
+    <col min="2" max="2" width="26.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
@@ -406,65 +490,265 @@
       <c r="A2" t="s">
         <v>2</v>
       </c>
+      <c r="B2" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>13</v>
       </c>
+      <c r="B3" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>3</v>
       </c>
+      <c r="B4" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>14</v>
       </c>
+      <c r="B5" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>4</v>
       </c>
+      <c r="B6" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>5</v>
       </c>
+      <c r="B7" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>11</v>
       </c>
+      <c r="B8" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>6</v>
       </c>
+      <c r="B9" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>7</v>
       </c>
+      <c r="B10" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>8</v>
       </c>
+      <c r="B11" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>9</v>
       </c>
+      <c r="B12" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>10</v>
       </c>
+      <c r="B13" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>12</v>
+      </c>
+      <c r="B14" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>15</v>
+      </c>
+      <c r="B15" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>16</v>
+      </c>
+      <c r="B16" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>17</v>
+      </c>
+      <c r="B17" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>28</v>
+      </c>
+      <c r="B18" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>27</v>
+      </c>
+      <c r="B19" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>21</v>
+      </c>
+      <c r="B20" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>22</v>
+      </c>
+      <c r="B21" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>23</v>
+      </c>
+      <c r="B22" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>24</v>
+      </c>
+      <c r="B23" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>25</v>
+      </c>
+      <c r="B24" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>26</v>
+      </c>
+      <c r="B25" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>29</v>
+      </c>
+      <c r="B26" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>30</v>
+      </c>
+      <c r="B27" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>31</v>
+      </c>
+      <c r="B28" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>33</v>
+      </c>
+      <c r="B29" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>34</v>
+      </c>
+      <c r="B30" t="s">
+        <v>39</v>
+      </c>
+      <c r="E30" s="1"/>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>35</v>
+      </c>
+      <c r="B31" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>36</v>
+      </c>
+      <c r="B32" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>37</v>
+      </c>
+      <c r="B33" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
+        <v>38</v>
+      </c>
+      <c r="B34" t="s">
+        <v>39</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: PWA installable — manifest, service worker, install button in header
</commit_message>
<xml_diff>
--- a/public/clientes.xlsx
+++ b/public/clientes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yeres\OneDrive\Documentos\Webs\PREVENA PG\Skills\PreventaPG\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B006F855-34D4-4D6A-86A3-6F420B5EABAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2035AE2-92C8-4D1C-BFFF-45DC781BEF20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="41">
   <si>
     <t>Cliente</t>
   </si>
@@ -145,6 +145,9 @@
   </si>
   <si>
     <t>Talara - Parada</t>
+  </si>
+  <si>
+    <t>Prueba y tanteo</t>
   </si>
 </sst>
 </file>
@@ -188,9 +191,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -471,7 +475,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E34"/>
+  <dimension ref="A1:E36"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="35.33203125" customWidth="1"/>
@@ -751,6 +755,17 @@
         <v>39</v>
       </c>
     </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>40</v>
+      </c>
+      <c r="B35" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A36" s="2"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>